<commit_message>
Update working project files and add frontend workspace config
</commit_message>
<xml_diff>
--- a/tests/Data to recon/result.xlsx
+++ b/tests/Data to recon/result.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="01 Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="02 Exceptions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="03 Matched Records" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="04 Missing - RecliQ_Universal_R" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="05 Missing - RecliQ_Universal_R" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="06 Field Differences" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="07 Control Checks" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Exceptions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Matched Records" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Missing - RecliQ_Universal_R" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Missing - RecliQ_Universal_R" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Field Differences" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Control Checks" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02 Exceptions'!$A$4:$K$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02 Exceptions'!$A$4:$K$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -286,22 +286,22 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -427,13 +427,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -456,17 +456,17 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <dPt>
             <idx val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="1E7B34"/>
               </a:solidFill>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -474,10 +474,10 @@
           <dPt>
             <idx val="1"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B36A00"/>
               </a:solidFill>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -485,10 +485,10 @@
           <dPt>
             <idx val="2"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="A6192E"/>
               </a:solidFill>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -496,10 +496,10 @@
           <dPt>
             <idx val="3"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="7A0C1E"/>
               </a:solidFill>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -529,14 +529,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -560,21 +560,21 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1F3864"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'01 Executive Summary'!$B$26:$B$30</f>
+              <f>'01 Executive Summary'!$B$26:$B$31</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'01 Executive Summary'!$D$26:$D$30</f>
+              <f>'01 Executive Summary'!$D$26:$D$31</f>
             </numRef>
           </val>
         </ser>
@@ -612,7 +612,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -627,9 +627,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -649,9 +649,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -661,37 +661,55 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Missing_04MissingRecliQ_Univer" displayName="Missing_04MissingRecliQ_Univer" ref="A4:J6" headerRowCount="1">
-  <autoFilter ref="A4:J6"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="DOCUMENT NUMBER"/>
-    <tableColumn id="2" name="POSTING DATE"/>
-    <tableColumn id="3" name="SUPPLIER"/>
-    <tableColumn id="4" name="BASE AMOUNT"/>
-    <tableColumn id="5" name="TAX AMOUNT"/>
-    <tableColumn id="6" name="GROSS AMOUNT"/>
-    <tableColumn id="7" name="STATUS"/>
-    <tableColumn id="8" name="PORTAL REFERENCE"/>
-    <tableColumn id="9" name="CATEGORY"/>
-    <tableColumn id="10" name="RecliQ_Universal_Reconciliation_Master_Test - portal.xlsx Row"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Missing_04MissingRecliQ_Univer" displayName="Missing_04MissingRecliQ_Univer" ref="A4:S8" headerRowCount="1">
+  <autoFilter ref="A4:S8"/>
+  <tableColumns count="19">
+    <tableColumn id="1" name="NORM_DOCUMENT NUMBER"/>
+    <tableColumn id="2" name="BASE AMOUNT"/>
+    <tableColumn id="3" name="GROSS AMOUNT"/>
+    <tableColumn id="4" name="DOCUMENT NUMBER"/>
+    <tableColumn id="5" name="POSTING DATE"/>
+    <tableColumn id="6" name="SUPPLIER"/>
+    <tableColumn id="7" name="TAX AMOUNT"/>
+    <tableColumn id="8" name="STATUS"/>
+    <tableColumn id="9" name="PORTAL REFERENCE"/>
+    <tableColumn id="10" name="CATEGORY"/>
+    <tableColumn id="11" name="__SOURCE_FILE__"/>
+    <tableColumn id="12" name="__SOURCE_SHEET__"/>
+    <tableColumn id="13" name="__SOURCE_ROW__"/>
+    <tableColumn id="14" name="NORM_POSTING DATE"/>
+    <tableColumn id="15" name="NORM_SUPPLIER"/>
+    <tableColumn id="16" name="NORM_BASE AMOUNT"/>
+    <tableColumn id="17" name="NORM_GROSS AMOUNT"/>
+    <tableColumn id="18" name="__GROUP_COUNT__"/>
+    <tableColumn id="19" name="RecliQ_Universal_Reconciliation_Master_Test - portal.xlsx Row"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Missing_05MissingRecliQ_Univer" displayName="Missing_05MissingRecliQ_Univer" ref="A4:I6" headerRowCount="1">
-  <autoFilter ref="A4:I6"/>
-  <tableColumns count="9">
-    <tableColumn id="1" name="INVOICE NO"/>
-    <tableColumn id="2" name="INVOICE DATE"/>
-    <tableColumn id="3" name="VENDOR NAME"/>
-    <tableColumn id="4" name="TAXABLE VALUE"/>
-    <tableColumn id="5" name="GST"/>
-    <tableColumn id="6" name="TOTAL BOOK VALUE"/>
-    <tableColumn id="7" name="DEPARTMENT"/>
-    <tableColumn id="8" name="PO REFERENCE"/>
-    <tableColumn id="9" name="RecliQ_Universal_Reconciliation_Master_Test - Book.xlsx Row"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Missing_05MissingRecliQ_Univer" displayName="Missing_05MissingRecliQ_Univer" ref="A4:R6" headerRowCount="1">
+  <autoFilter ref="A4:R6"/>
+  <tableColumns count="18">
+    <tableColumn id="1" name="NORM_INVOICE NO"/>
+    <tableColumn id="2" name="TAXABLE VALUE"/>
+    <tableColumn id="3" name="TOTAL BOOK VALUE"/>
+    <tableColumn id="4" name="INVOICE NO"/>
+    <tableColumn id="5" name="INVOICE DATE"/>
+    <tableColumn id="6" name="VENDOR NAME"/>
+    <tableColumn id="7" name="GST"/>
+    <tableColumn id="8" name="DEPARTMENT"/>
+    <tableColumn id="9" name="PO REFERENCE"/>
+    <tableColumn id="10" name="__SOURCE_FILE__"/>
+    <tableColumn id="11" name="__SOURCE_SHEET__"/>
+    <tableColumn id="12" name="__SOURCE_ROW__"/>
+    <tableColumn id="13" name="NORM_INVOICE DATE"/>
+    <tableColumn id="14" name="NORM_VENDOR NAME"/>
+    <tableColumn id="15" name="NORM_TAXABLE VALUE"/>
+    <tableColumn id="16" name="NORM_TOTAL BOOK VALUE"/>
+    <tableColumn id="17" name="__GROUP_COUNT__"/>
+    <tableColumn id="18" name="RecliQ_Universal_Reconciliation_Master_Test - Book.xlsx Row"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -987,7 +1005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:N44"/>
+  <dimension ref="B1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.44" customWidth="1" min="1" max="1"/>
@@ -1067,7 +1085,7 @@
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="B6" s="6">
-        <f>COUNTA('03 Matched Records'!C5:C5)+SUM('02 Exceptions'!L5:L20)+COUNTA('04 Missing - RecliQ_Universal_R'!A5:A6)+COUNTA('05 Missing - RecliQ_Universal_R'!A5:A6)</f>
+        <f>COUNTA('03 Matched Records'!C5:C5)+SUM('02 Exceptions'!L5:L38)+COUNTA('04 Missing - RecliQ_Universal_R'!A5:A8)+COUNTA('05 Missing - RecliQ_Universal_R'!A5:A6)</f>
         <v/>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -1077,12 +1095,12 @@
       </c>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="8">
-        <f>SUM('02 Exceptions'!L5:L20)</f>
+        <f>SUM('02 Exceptions'!L5:L38)</f>
         <v/>
       </c>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="9">
-        <f>COUNTA('04 Missing - RecliQ_Universal_R'!A5:A6)+COUNTA('05 Missing - RecliQ_Universal_R'!A5:A6)</f>
+        <f>COUNTA('04 Missing - RecliQ_Universal_R'!A5:A8)+COUNTA('05 Missing - RecliQ_Universal_R'!A5:A6)</f>
         <v/>
       </c>
       <c r="I6" s="5" t="n"/>
@@ -1109,12 +1127,12 @@
       </c>
       <c r="E7" s="13" t="n"/>
       <c r="F7" s="12">
-        <f>(COUNTA('02 Exceptions'!B5:B20))&amp;" field-level mismatch(es)"</f>
+        <f>(COUNTA('02 Exceptions'!B5:B38))&amp;" field-level mismatch(es)"</f>
         <v/>
       </c>
       <c r="G7" s="13" t="n"/>
       <c r="H7" s="12">
-        <f>(COUNTA('04 Missing - RecliQ_Universal_R'!A5:A6))&amp;" + "&amp;(COUNTA('05 Missing - RecliQ_Universal_R'!A5:A6))&amp;" by source"</f>
+        <f>(COUNTA('04 Missing - RecliQ_Universal_R'!A5:A8))&amp;" + "&amp;(COUNTA('05 Missing - RecliQ_Universal_R'!A5:A6))&amp;" by source"</f>
         <v/>
       </c>
       <c r="I7" s="13" t="n"/>
@@ -1190,7 +1208,7 @@
         </is>
       </c>
       <c r="C13" s="16">
-        <f>COUNTA('04 Missing - RecliQ_Universal_R'!A5:A6)</f>
+        <f>COUNTA('04 Missing - RecliQ_Universal_R'!A5:A8)</f>
         <v/>
       </c>
       <c r="D13" s="17">
@@ -1259,7 +1277,7 @@
         </is>
       </c>
       <c r="C19" s="16">
-        <f>COUNTIFS('02 Exceptions'!$H$5:$H$20,"Value Difference")</f>
+        <f>COUNTIFS('02 Exceptions'!$H$5:$H$38,"Value Difference")</f>
         <v/>
       </c>
       <c r="D19" s="17">
@@ -1274,7 +1292,7 @@
         </is>
       </c>
       <c r="C20" s="19">
-        <f>COUNTIFS('02 Exceptions'!$H$5:$H$20,"Text Difference")</f>
+        <f>COUNTIFS('02 Exceptions'!$H$5:$H$38,"Text Difference")</f>
         <v/>
       </c>
       <c r="D20" s="20">
@@ -1289,7 +1307,7 @@
         </is>
       </c>
       <c r="C21" s="16">
-        <f>COUNTA('04 Missing - RecliQ_Universal_R'!A5:A6)</f>
+        <f>COUNTA('04 Missing - RecliQ_Universal_R'!A5:A8)</f>
         <v/>
       </c>
       <c r="D21" s="17">
@@ -1344,7 +1362,7 @@
     <row r="26">
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>GST</t>
+          <t>VENDOR NAME</t>
         </is>
       </c>
       <c r="C26" s="16">
@@ -1352,7 +1370,7 @@
         <v/>
       </c>
       <c r="D26" s="16">
-        <f>COUNTIFS('02 Exceptions'!$C$5:$C$20,B26)</f>
+        <f>COUNTIFS('02 Exceptions'!$C$5:$C$38,B26)</f>
         <v/>
       </c>
       <c r="E26" s="17">
@@ -1363,7 +1381,7 @@
     <row r="27">
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>VENDOR NAME</t>
+          <t>TAXABLE VALUE</t>
         </is>
       </c>
       <c r="C27" s="19">
@@ -1371,7 +1389,7 @@
         <v/>
       </c>
       <c r="D27" s="19">
-        <f>COUNTIFS('02 Exceptions'!$C$5:$C$20,B27)</f>
+        <f>COUNTIFS('02 Exceptions'!$C$5:$C$38,B27)</f>
         <v/>
       </c>
       <c r="E27" s="20">
@@ -1382,7 +1400,7 @@
     <row r="28">
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>TAXABLE VALUE</t>
+          <t>GST</t>
         </is>
       </c>
       <c r="C28" s="16">
@@ -1390,7 +1408,7 @@
         <v/>
       </c>
       <c r="D28" s="16">
-        <f>COUNTIFS('02 Exceptions'!$C$5:$C$20,B28)</f>
+        <f>COUNTIFS('02 Exceptions'!$C$5:$C$38,B28)</f>
         <v/>
       </c>
       <c r="E28" s="17">
@@ -1409,7 +1427,7 @@
         <v/>
       </c>
       <c r="D29" s="19">
-        <f>COUNTIFS('02 Exceptions'!$C$5:$C$20,B29)</f>
+        <f>COUNTIFS('02 Exceptions'!$C$5:$C$38,B29)</f>
         <v/>
       </c>
       <c r="E29" s="20">
@@ -1428,7 +1446,7 @@
         <v/>
       </c>
       <c r="D30" s="16">
-        <f>COUNTIFS('02 Exceptions'!$C$5:$C$20,B30)</f>
+        <f>COUNTIFS('02 Exceptions'!$C$5:$C$38,B30)</f>
         <v/>
       </c>
       <c r="E30" s="17">
@@ -1436,110 +1454,129 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="21.75" customHeight="1">
-      <c r="B32" s="3" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C31" s="19">
+        <f>$D$6</f>
+        <v/>
+      </c>
+      <c r="D31" s="19">
+        <f>COUNTIFS('02 Exceptions'!$C$5:$C$38,B31)</f>
+        <v/>
+      </c>
+      <c r="E31" s="20">
+        <f>IF((C31+D31)&gt;0,C31/(C31+D31),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="21.75" customHeight="1">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>KEY INSIGHTS</t>
         </is>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="B33" s="24">
-        <f>"•  "&amp;TEXT($J$6,"0.0%")&amp;" of records matched perfectly ("&amp;$D$6&amp;" of "&amp;$B$6&amp;")."</f>
-        <v/>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="B34" s="24">
-        <f>"•  "&amp;$F$6&amp;" discrepant record(s) identified ("&amp;(COUNTA('02 Exceptions'!B5:B20))&amp;" field mismatches) — review required."</f>
+        <f>"•  "&amp;TEXT($J$6,"0.0%")&amp;" of records matched perfectly ("&amp;$D$6&amp;" of "&amp;$B$6&amp;")."</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="B35" s="24">
-        <f>"•  "&amp;(COUNTA('04 Missing - RecliQ_Universal_R'!A5:A6)+COUNTA('05 Missing - RecliQ_Universal_R'!A5:A6))&amp;" record(s) missing from one or both sources ("&amp;(COUNTA('04 Missing - RecliQ_Universal_R'!A5:A6))&amp;" RecliQ_Universal_Reconciliation_Master_Test - Book.xlsx, "&amp;(COUNTA('05 Missing - RecliQ_Universal_R'!A5:A6))&amp;" RecliQ_Universal_Reconciliation_Master_Test - portal.xlsx)."</f>
+        <f>"•  "&amp;$F$6&amp;" discrepant record(s) identified ("&amp;(COUNTA('02 Exceptions'!B5:B38))&amp;" field mismatches) — review required."</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="B36" s="24">
-        <f>"•  Field '"&amp;INDEX($B$26:$B$30,MATCH(MAX($D$26:$D$30),$D$26:$D$30,0))&amp;"' has the highest exception count ("&amp;MAX($D$26:$D$30)&amp;")."</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="21.75" customHeight="1">
-      <c r="B38" s="3" t="inlineStr">
+        <f>"•  "&amp;(COUNTA('04 Missing - RecliQ_Universal_R'!A5:A8)+COUNTA('05 Missing - RecliQ_Universal_R'!A5:A6))&amp;" record(s) missing from one or both sources ("&amp;(COUNTA('04 Missing - RecliQ_Universal_R'!A5:A8))&amp;" RecliQ_Universal_Reconciliation_Master_Test - Book.xlsx, "&amp;(COUNTA('05 Missing - RecliQ_Universal_R'!A5:A6))&amp;" RecliQ_Universal_Reconciliation_Master_Test - portal.xlsx)."</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="B37" s="24">
+        <f>"•  Field '"&amp;INDEX($B$26:$B$31,MATCH(MAX($D$26:$D$31),$D$26:$D$31,0))&amp;"' has the highest exception count ("&amp;MAX($D$26:$D$31)&amp;")."</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="21.75" customHeight="1">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>CONTROL SUMMARY</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="15.75" customHeight="1">
-      <c r="B39" s="4" t="inlineStr">
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>Total Records</t>
         </is>
-      </c>
-      <c r="C39" s="5" t="n"/>
-      <c r="D39" s="5" t="n"/>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>Outstanding Exceptions</t>
-        </is>
-      </c>
-      <c r="F39" s="5" t="n"/>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>Missing Records</t>
-        </is>
-      </c>
-      <c r="I39" s="5" t="n"/>
-      <c r="J39" s="5" t="n"/>
-      <c r="K39" s="4" t="inlineStr">
-        <is>
-          <t>Full Audit Trail</t>
-        </is>
-      </c>
-      <c r="L39" s="5" t="n"/>
-      <c r="M39" s="5" t="n"/>
-    </row>
-    <row r="40" ht="21.75" customHeight="1">
-      <c r="B40" s="25">
-        <f>$B$6</f>
-        <v/>
       </c>
       <c r="C40" s="5" t="n"/>
       <c r="D40" s="5" t="n"/>
-      <c r="E40" s="25">
-        <f>$F$6</f>
-        <v/>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Outstanding Exceptions</t>
+        </is>
       </c>
       <c r="F40" s="5" t="n"/>
       <c r="G40" s="5" t="n"/>
-      <c r="H40" s="25">
-        <f>$H$6</f>
-        <v/>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>Missing Records</t>
+        </is>
       </c>
       <c r="I40" s="5" t="n"/>
       <c r="J40" s="5" t="n"/>
-      <c r="K40" s="26" t="inlineStr">
-        <is>
-          <t>See tab 07</t>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>Full Audit Trail</t>
         </is>
       </c>
       <c r="L40" s="5" t="n"/>
       <c r="M40" s="5" t="n"/>
     </row>
-    <row r="42">
-      <c r="B42" s="27" t="inlineStr">
+    <row r="41" ht="21.75" customHeight="1">
+      <c r="B41" s="25">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="25">
+        <f>$F$6</f>
+        <v/>
+      </c>
+      <c r="F41" s="5" t="n"/>
+      <c r="G41" s="5" t="n"/>
+      <c r="H41" s="25">
+        <f>$H$6</f>
+        <v/>
+      </c>
+      <c r="I41" s="5" t="n"/>
+      <c r="J41" s="5" t="n"/>
+      <c r="K41" s="26" t="inlineStr">
+        <is>
+          <t>See tab 07</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="n"/>
+      <c r="M41" s="5" t="n"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="27" t="inlineStr">
         <is>
           <t>Full detail, formulas, and audit trail for every figure above are available on tabs 02–07 of this workbook.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="28" t="inlineStr">
+    <row r="45">
+      <c r="B45" s="28" t="inlineStr">
         <is>
           <t>RecliQ Reconciliation Engine  •  Confidential — Internal Use Only</t>
         </is>
@@ -1547,32 +1584,33 @@
     </row>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="B37:N37"/>
+    <mergeCell ref="K41:M41"/>
     <mergeCell ref="L7:M7"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="J5:K5"/>
-    <mergeCell ref="B42:M42"/>
     <mergeCell ref="K40:M40"/>
     <mergeCell ref="E40:G40"/>
     <mergeCell ref="F6:G6"/>
-    <mergeCell ref="B33:N33"/>
-    <mergeCell ref="B44:M44"/>
     <mergeCell ref="F7:G7"/>
+    <mergeCell ref="B43:M43"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="B36:N36"/>
-    <mergeCell ref="B38:M38"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="B35:N35"/>
     <mergeCell ref="B4:N4"/>
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="B40:D40"/>
-    <mergeCell ref="K39:M39"/>
     <mergeCell ref="L5:M5"/>
     <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B33:M33"/>
     <mergeCell ref="D7:E7"/>
+    <mergeCell ref="E41:G41"/>
+    <mergeCell ref="B41:D41"/>
     <mergeCell ref="H7:I7"/>
+    <mergeCell ref="B45:M45"/>
     <mergeCell ref="J7:K7"/>
-    <mergeCell ref="B32:M32"/>
     <mergeCell ref="B2:N2"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B6:C6"/>
@@ -1580,13 +1618,12 @@
     <mergeCell ref="L6:M6"/>
     <mergeCell ref="B1:N1"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="E39:G39"/>
+    <mergeCell ref="H41:J41"/>
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="H40:J40"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="H39:J39"/>
     <mergeCell ref="B34:N34"/>
+    <mergeCell ref="B39:M39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1600,7 +1637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.5" customWidth="1" min="1" max="1"/>
@@ -1696,39 +1733,37 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>EX-000002</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>INV/1002</t>
-        </is>
-      </c>
+          <t>EX-000001</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr"/>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>INVOICE DATE</t>
+          <t>PO REFERENCE</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>02-Aug-2026</t>
+          <t>PO-501</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="F5" s="31" t="n"/>
-      <c r="G5" s="31" t="n"/>
+          <t>P-9001</t>
+        </is>
+      </c>
+      <c r="F5" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G5" s="32" t="n"/>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>Text Difference</t>
+          <t>Value Difference</t>
         </is>
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J5" s="15" t="inlineStr">
@@ -1737,7 +1772,7 @@
         </is>
       </c>
       <c r="K5" s="15" t="inlineStr"/>
-      <c r="L5" s="31">
+      <c r="L5" s="32">
         <f>IF(COUNTIF($B$5:B5,B5)=1,1,0)</f>
         <v/>
       </c>
@@ -1745,14 +1780,10 @@
     <row r="6">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>EX-000004</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>INV/1004</t>
-        </is>
-      </c>
+          <t>EX-000002</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr"/>
       <c r="C6" s="18" t="inlineStr">
         <is>
           <t>INVOICE DATE</t>
@@ -1760,26 +1791,24 @@
       </c>
       <c r="D6" s="18" t="inlineStr">
         <is>
-          <t>2026/08/04</t>
+          <t>02-Aug-2026</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
         <is>
-          <t>04/08/2026</t>
-        </is>
-      </c>
-      <c r="F6" s="32" t="n">
-        <v>16178778</v>
-      </c>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="F6" s="33" t="n"/>
       <c r="G6" s="33" t="n"/>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>Value Difference</t>
+          <t>Text Difference</t>
         </is>
       </c>
       <c r="I6" s="18" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J6" s="18" t="inlineStr">
@@ -1796,39 +1825,37 @@
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>EX-000005</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="inlineStr">
-        <is>
-          <t>INV/1005</t>
-        </is>
-      </c>
+          <t>EX-000002</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr"/>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>INVOICE DATE</t>
+          <t>PO REFERENCE</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>05-08-2026</t>
+          <t>PO-502</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="F7" s="31" t="n"/>
-      <c r="G7" s="31" t="n"/>
+          <t>P-9002</t>
+        </is>
+      </c>
+      <c r="F7" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G7" s="32" t="n"/>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>Text Difference</t>
+          <t>Value Difference</t>
         </is>
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J7" s="15" t="inlineStr">
@@ -1837,7 +1864,7 @@
         </is>
       </c>
       <c r="K7" s="15" t="inlineStr"/>
-      <c r="L7" s="31">
+      <c r="L7" s="32">
         <f>IF(COUNTIF($B$5:B7,B7)=1,1,0)</f>
         <v/>
       </c>
@@ -1845,39 +1872,37 @@
     <row r="8">
       <c r="A8" s="18" t="inlineStr">
         <is>
-          <t>EX-000006</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>INV/1006</t>
-        </is>
-      </c>
+          <t>EX-000003</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr"/>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>INVOICE DATE</t>
+          <t>PO REFERENCE</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>PO-503</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>06-Aug-2026</t>
-        </is>
-      </c>
-      <c r="F8" s="33" t="n"/>
+          <t>P-9003</t>
+        </is>
+      </c>
+      <c r="F8" s="34" t="n">
+        <v>8500</v>
+      </c>
       <c r="G8" s="33" t="n"/>
       <c r="H8" s="18" t="inlineStr">
         <is>
-          <t>Text Difference</t>
+          <t>Value Difference</t>
         </is>
       </c>
       <c r="I8" s="18" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J8" s="18" t="inlineStr">
@@ -1894,14 +1919,10 @@
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>EX-000007</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>INV/1007</t>
-        </is>
-      </c>
+          <t>EX-000004</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr"/>
       <c r="C9" s="15" t="inlineStr">
         <is>
           <t>INVOICE DATE</t>
@@ -1909,18 +1930,18 @@
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>2026/08/04</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>2026/08/07</t>
-        </is>
-      </c>
-      <c r="F9" s="34" t="n">
-        <v>-13178781</v>
-      </c>
-      <c r="G9" s="31" t="n"/>
+          <t>04/08/2026</t>
+        </is>
+      </c>
+      <c r="F9" s="31" t="n">
+        <v>16178778</v>
+      </c>
+      <c r="G9" s="32" t="n"/>
       <c r="H9" s="15" t="inlineStr">
         <is>
           <t>Value Difference</t>
@@ -1937,7 +1958,7 @@
         </is>
       </c>
       <c r="K9" s="15" t="inlineStr"/>
-      <c r="L9" s="31">
+      <c r="L9" s="32">
         <f>IF(COUNTIF($B$5:B9,B9)=1,1,0)</f>
         <v/>
       </c>
@@ -1945,39 +1966,37 @@
     <row r="10">
       <c r="A10" s="18" t="inlineStr">
         <is>
-          <t>EX-000008</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>INV/1008</t>
-        </is>
-      </c>
+          <t>EX-000004</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr"/>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>INVOICE DATE</t>
+          <t>PO REFERENCE</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>PO-504</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>08-08-2026</t>
-        </is>
-      </c>
-      <c r="F10" s="33" t="n"/>
+          <t>P-9004</t>
+        </is>
+      </c>
+      <c r="F10" s="34" t="n">
+        <v>8500</v>
+      </c>
       <c r="G10" s="33" t="n"/>
       <c r="H10" s="18" t="inlineStr">
         <is>
-          <t>Text Difference</t>
+          <t>Value Difference</t>
         </is>
       </c>
       <c r="I10" s="18" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J10" s="18" t="inlineStr">
@@ -1994,14 +2013,10 @@
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>EX-000009</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="inlineStr">
-        <is>
-          <t>INV/1009</t>
-        </is>
-      </c>
+          <t>EX-000005</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr"/>
       <c r="C11" s="15" t="inlineStr">
         <is>
           <t>INVOICE DATE</t>
@@ -2009,16 +2024,16 @@
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>09-Aug-2026</t>
+          <t>05-08-2026</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="F11" s="31" t="n"/>
-      <c r="G11" s="31" t="n"/>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="F11" s="32" t="n"/>
+      <c r="G11" s="32" t="n"/>
       <c r="H11" s="15" t="inlineStr">
         <is>
           <t>Text Difference</t>
@@ -2035,7 +2050,7 @@
         </is>
       </c>
       <c r="K11" s="15" t="inlineStr"/>
-      <c r="L11" s="31">
+      <c r="L11" s="32">
         <f>IF(COUNTIF($B$5:B11,B11)=1,1,0)</f>
         <v/>
       </c>
@@ -2043,39 +2058,37 @@
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>EX-000012</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>INV/1012</t>
-        </is>
-      </c>
+          <t>EX-000005</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr"/>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>INVOICE DATE</t>
+          <t>PO REFERENCE</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>PO-505</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>12-Aug-2026</t>
-        </is>
-      </c>
-      <c r="F12" s="33" t="n"/>
+          <t>P-9005</t>
+        </is>
+      </c>
+      <c r="F12" s="34" t="n">
+        <v>8500</v>
+      </c>
       <c r="G12" s="33" t="n"/>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>Text Difference</t>
+          <t>Value Difference</t>
         </is>
       </c>
       <c r="I12" s="18" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J12" s="18" t="inlineStr">
@@ -2092,14 +2105,10 @@
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>EX-000017</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="inlineStr">
-        <is>
-          <t>INV/1017</t>
-        </is>
-      </c>
+          <t>EX-000006</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr"/>
       <c r="C13" s="15" t="inlineStr">
         <is>
           <t>INVOICE DATE</t>
@@ -2107,16 +2116,16 @@
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>17-Aug-2026</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="F13" s="31" t="n"/>
-      <c r="G13" s="31" t="n"/>
+          <t>06-Aug-2026</t>
+        </is>
+      </c>
+      <c r="F13" s="32" t="n"/>
+      <c r="G13" s="32" t="n"/>
       <c r="H13" s="15" t="inlineStr">
         <is>
           <t>Text Difference</t>
@@ -2133,7 +2142,7 @@
         </is>
       </c>
       <c r="K13" s="15" t="inlineStr"/>
-      <c r="L13" s="31">
+      <c r="L13" s="32">
         <f>IF(COUNTIF($B$5:B13,B13)=1,1,0)</f>
         <v/>
       </c>
@@ -2141,39 +2150,37 @@
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>EX-000019</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>INV/1020</t>
-        </is>
-      </c>
+          <t>EX-000006</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr"/>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>INVOICE DATE</t>
+          <t>PO REFERENCE</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>PO-506</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>20-Aug-2026</t>
-        </is>
-      </c>
-      <c r="F14" s="33" t="n"/>
+          <t>P-9006</t>
+        </is>
+      </c>
+      <c r="F14" s="34" t="n">
+        <v>8500</v>
+      </c>
       <c r="G14" s="33" t="n"/>
       <c r="H14" s="18" t="inlineStr">
         <is>
-          <t>Text Difference</t>
+          <t>Value Difference</t>
         </is>
       </c>
       <c r="I14" s="18" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J14" s="18" t="inlineStr">
@@ -2190,31 +2197,29 @@
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>EX-000020</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="inlineStr">
-        <is>
-          <t>INV/1022</t>
-        </is>
-      </c>
+          <t>EX-000007</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr"/>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>TAXABLE VALUE</t>
-        </is>
-      </c>
-      <c r="D15" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="34" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F15" s="34" t="n">
-        <v>-4000</v>
-      </c>
-      <c r="G15" s="35" t="n">
-        <v>-1</v>
-      </c>
+          <t>INVOICE DATE</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>2026/08/07</t>
+        </is>
+      </c>
+      <c r="F15" s="31" t="n">
+        <v>-13178781</v>
+      </c>
+      <c r="G15" s="32" t="n"/>
       <c r="H15" s="15" t="inlineStr">
         <is>
           <t>Value Difference</t>
@@ -2231,7 +2236,7 @@
         </is>
       </c>
       <c r="K15" s="15" t="inlineStr"/>
-      <c r="L15" s="31">
+      <c r="L15" s="32">
         <f>IF(COUNTIF($B$5:B15,B15)=1,1,0)</f>
         <v/>
       </c>
@@ -2239,31 +2244,29 @@
     <row r="16">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t>EX-000020</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>INV/1022</t>
-        </is>
-      </c>
+          <t>EX-000007</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr"/>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>GST</t>
-        </is>
-      </c>
-      <c r="D16" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="32" t="n">
-        <v>720</v>
-      </c>
-      <c r="F16" s="32" t="n">
-        <v>-720</v>
-      </c>
-      <c r="G16" s="36" t="n">
-        <v>-1</v>
-      </c>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>PO-507</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>P-9007</t>
+        </is>
+      </c>
+      <c r="F16" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G16" s="33" t="n"/>
       <c r="H16" s="18" t="inlineStr">
         <is>
           <t>Value Difference</t>
@@ -2271,7 +2274,7 @@
       </c>
       <c r="I16" s="18" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J16" s="18" t="inlineStr">
@@ -2288,39 +2291,35 @@
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>EX-000020</t>
-        </is>
-      </c>
-      <c r="B17" s="15" t="inlineStr">
-        <is>
-          <t>INV/1022</t>
-        </is>
-      </c>
+          <t>EX-000008</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr"/>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>TOTAL BOOK VALUE</t>
-        </is>
-      </c>
-      <c r="D17" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="34" t="n">
-        <v>4720</v>
-      </c>
-      <c r="F17" s="34" t="n">
-        <v>-4720</v>
-      </c>
-      <c r="G17" s="35" t="n">
-        <v>-1</v>
-      </c>
+          <t>INVOICE DATE</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>08-08-2026</t>
+        </is>
+      </c>
+      <c r="F17" s="32" t="n"/>
+      <c r="G17" s="32" t="n"/>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>Value Difference</t>
+          <t>Text Difference</t>
         </is>
       </c>
       <c r="I17" s="15" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J17" s="15" t="inlineStr">
@@ -2329,7 +2328,7 @@
         </is>
       </c>
       <c r="K17" s="15" t="inlineStr"/>
-      <c r="L17" s="31">
+      <c r="L17" s="32">
         <f>IF(COUNTIF($B$5:B17,B17)=1,1,0)</f>
         <v/>
       </c>
@@ -2337,31 +2336,29 @@
     <row r="18">
       <c r="A18" s="18" t="inlineStr">
         <is>
-          <t>EX-000021</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>INV/1023</t>
-        </is>
-      </c>
+          <t>EX-000008</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr"/>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>TAXABLE VALUE</t>
-        </is>
-      </c>
-      <c r="D18" s="32" t="n">
-        <v>12000</v>
-      </c>
-      <c r="E18" s="32" t="n">
-        <v>24000</v>
-      </c>
-      <c r="F18" s="32" t="n">
-        <v>-12000</v>
-      </c>
-      <c r="G18" s="36" t="n">
-        <v>-0.5</v>
-      </c>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>PO-508</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>P-9008</t>
+        </is>
+      </c>
+      <c r="F18" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G18" s="33" t="n"/>
       <c r="H18" s="18" t="inlineStr">
         <is>
           <t>Value Difference</t>
@@ -2386,39 +2383,35 @@
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>EX-000021</t>
-        </is>
-      </c>
-      <c r="B19" s="15" t="inlineStr">
-        <is>
-          <t>INV/1023</t>
-        </is>
-      </c>
+          <t>EX-000009</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr"/>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>GST</t>
-        </is>
-      </c>
-      <c r="D19" s="34" t="n">
-        <v>2160</v>
-      </c>
-      <c r="E19" s="34" t="n">
-        <v>4320</v>
-      </c>
-      <c r="F19" s="34" t="n">
-        <v>-2160</v>
-      </c>
-      <c r="G19" s="35" t="n">
-        <v>-0.5</v>
-      </c>
+          <t>INVOICE DATE</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>09-Aug-2026</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="F19" s="32" t="n"/>
+      <c r="G19" s="32" t="n"/>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>Value Difference</t>
+          <t>Text Difference</t>
         </is>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J19" s="15" t="inlineStr">
@@ -2427,7 +2420,7 @@
         </is>
       </c>
       <c r="K19" s="15" t="inlineStr"/>
-      <c r="L19" s="31">
+      <c r="L19" s="32">
         <f>IF(COUNTIF($B$5:B19,B19)=1,1,0)</f>
         <v/>
       </c>
@@ -2435,31 +2428,29 @@
     <row r="20">
       <c r="A20" s="18" t="inlineStr">
         <is>
-          <t>EX-000021</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>INV/1023</t>
-        </is>
-      </c>
+          <t>EX-000009</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr"/>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>TOTAL BOOK VALUE</t>
-        </is>
-      </c>
-      <c r="D20" s="32" t="n">
-        <v>14160</v>
-      </c>
-      <c r="E20" s="32" t="n">
-        <v>28320</v>
-      </c>
-      <c r="F20" s="32" t="n">
-        <v>-14160</v>
-      </c>
-      <c r="G20" s="36" t="n">
-        <v>-0.5</v>
-      </c>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>PO-509</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>P-9009</t>
+        </is>
+      </c>
+      <c r="F20" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G20" s="33" t="n"/>
       <c r="H20" s="18" t="inlineStr">
         <is>
           <t>Value Difference</t>
@@ -2481,8 +2472,842 @@
         <v/>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>EX-000010</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr"/>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>PO-510</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>P-9010</t>
+        </is>
+      </c>
+      <c r="F21" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G21" s="32" t="n"/>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I21" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J21" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K21" s="15" t="inlineStr"/>
+      <c r="L21" s="32">
+        <f>IF(COUNTIF($B$5:B21,B21)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>EX-000011</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr"/>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>PO-511</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>P-9011</t>
+        </is>
+      </c>
+      <c r="F22" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G22" s="33" t="n"/>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I22" s="18" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J22" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K22" s="18" t="inlineStr"/>
+      <c r="L22" s="33">
+        <f>IF(COUNTIF($B$5:B22,B22)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>EX-000012</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr"/>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>INVOICE DATE</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>12-Aug-2026</t>
+        </is>
+      </c>
+      <c r="F23" s="32" t="n"/>
+      <c r="G23" s="32" t="n"/>
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>Text Difference</t>
+        </is>
+      </c>
+      <c r="I23" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J23" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K23" s="15" t="inlineStr"/>
+      <c r="L23" s="32">
+        <f>IF(COUNTIF($B$5:B23,B23)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>EX-000012</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr"/>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>PO-512</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>P-9012</t>
+        </is>
+      </c>
+      <c r="F24" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G24" s="33" t="n"/>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J24" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K24" s="18" t="inlineStr"/>
+      <c r="L24" s="33">
+        <f>IF(COUNTIF($B$5:B24,B24)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>EX-000013</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="inlineStr"/>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>PO-513</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>P-9013</t>
+        </is>
+      </c>
+      <c r="F25" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G25" s="32" t="n"/>
+      <c r="H25" s="15" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I25" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J25" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K25" s="15" t="inlineStr"/>
+      <c r="L25" s="32">
+        <f>IF(COUNTIF($B$5:B25,B25)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>EX-000014</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr"/>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>PO-514</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>P-9014</t>
+        </is>
+      </c>
+      <c r="F26" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G26" s="33" t="n"/>
+      <c r="H26" s="18" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I26" s="18" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J26" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K26" s="18" t="inlineStr"/>
+      <c r="L26" s="33">
+        <f>IF(COUNTIF($B$5:B26,B26)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>EX-000015</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="inlineStr"/>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>PO-515</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>P-9015</t>
+        </is>
+      </c>
+      <c r="F27" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G27" s="32" t="n"/>
+      <c r="H27" s="15" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I27" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J27" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K27" s="15" t="inlineStr"/>
+      <c r="L27" s="32">
+        <f>IF(COUNTIF($B$5:B27,B27)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>EX-000016</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr"/>
+      <c r="C28" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>PO-516</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>P-9016</t>
+        </is>
+      </c>
+      <c r="F28" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G28" s="33" t="n"/>
+      <c r="H28" s="18" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I28" s="18" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J28" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K28" s="18" t="inlineStr"/>
+      <c r="L28" s="33">
+        <f>IF(COUNTIF($B$5:B28,B28)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>EX-000017</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr"/>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>INVOICE DATE</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>17-Aug-2026</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="F29" s="32" t="n"/>
+      <c r="G29" s="32" t="n"/>
+      <c r="H29" s="15" t="inlineStr">
+        <is>
+          <t>Text Difference</t>
+        </is>
+      </c>
+      <c r="I29" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J29" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K29" s="15" t="inlineStr"/>
+      <c r="L29" s="32">
+        <f>IF(COUNTIF($B$5:B29,B29)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>EX-000017</t>
+        </is>
+      </c>
+      <c r="B30" s="18" t="inlineStr"/>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>PO-517</t>
+        </is>
+      </c>
+      <c r="E30" s="18" t="inlineStr">
+        <is>
+          <t>P-9017</t>
+        </is>
+      </c>
+      <c r="F30" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G30" s="33" t="n"/>
+      <c r="H30" s="18" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I30" s="18" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J30" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K30" s="18" t="inlineStr"/>
+      <c r="L30" s="33">
+        <f>IF(COUNTIF($B$5:B30,B30)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>EX-000018</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="inlineStr"/>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>PO-518</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="inlineStr">
+        <is>
+          <t>P-9018</t>
+        </is>
+      </c>
+      <c r="F31" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G31" s="32" t="n"/>
+      <c r="H31" s="15" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I31" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J31" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K31" s="15" t="inlineStr"/>
+      <c r="L31" s="32">
+        <f>IF(COUNTIF($B$5:B31,B31)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>EX-000019</t>
+        </is>
+      </c>
+      <c r="B32" s="18" t="inlineStr"/>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>INVOICE DATE</t>
+        </is>
+      </c>
+      <c r="D32" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="E32" s="18" t="inlineStr">
+        <is>
+          <t>20-Aug-2026</t>
+        </is>
+      </c>
+      <c r="F32" s="33" t="n"/>
+      <c r="G32" s="33" t="n"/>
+      <c r="H32" s="18" t="inlineStr">
+        <is>
+          <t>Text Difference</t>
+        </is>
+      </c>
+      <c r="I32" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J32" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K32" s="18" t="inlineStr"/>
+      <c r="L32" s="33">
+        <f>IF(COUNTIF($B$5:B32,B32)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>EX-000019</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="inlineStr"/>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>PO-520</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>P-9020</t>
+        </is>
+      </c>
+      <c r="F33" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G33" s="32" t="n"/>
+      <c r="H33" s="15" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I33" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J33" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K33" s="15" t="inlineStr"/>
+      <c r="L33" s="32">
+        <f>IF(COUNTIF($B$5:B33,B33)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>EX-000020</t>
+        </is>
+      </c>
+      <c r="B34" s="18" t="inlineStr"/>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>TAXABLE VALUE</t>
+        </is>
+      </c>
+      <c r="D34" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="34" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F34" s="34" t="n">
+        <v>-4000</v>
+      </c>
+      <c r="G34" s="35" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H34" s="18" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I34" s="18" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J34" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K34" s="18" t="inlineStr"/>
+      <c r="L34" s="33">
+        <f>IF(COUNTIF($B$5:B34,B34)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>EX-000020</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="inlineStr"/>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>GST</t>
+        </is>
+      </c>
+      <c r="D35" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="31" t="n">
+        <v>720</v>
+      </c>
+      <c r="F35" s="31" t="n">
+        <v>-720</v>
+      </c>
+      <c r="G35" s="36" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H35" s="15" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I35" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J35" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K35" s="15" t="inlineStr"/>
+      <c r="L35" s="32">
+        <f>IF(COUNTIF($B$5:B35,B35)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="18" t="inlineStr">
+        <is>
+          <t>EX-000020</t>
+        </is>
+      </c>
+      <c r="B36" s="18" t="inlineStr"/>
+      <c r="C36" s="18" t="inlineStr">
+        <is>
+          <t>TOTAL BOOK VALUE</t>
+        </is>
+      </c>
+      <c r="D36" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="34" t="n">
+        <v>4720</v>
+      </c>
+      <c r="F36" s="34" t="n">
+        <v>-4720</v>
+      </c>
+      <c r="G36" s="35" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H36" s="18" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I36" s="18" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J36" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K36" s="18" t="inlineStr"/>
+      <c r="L36" s="33">
+        <f>IF(COUNTIF($B$5:B36,B36)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
+        <is>
+          <t>EX-000020</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="inlineStr"/>
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>PO-522</t>
+        </is>
+      </c>
+      <c r="E37" s="15" t="inlineStr">
+        <is>
+          <t>P-9022</t>
+        </is>
+      </c>
+      <c r="F37" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G37" s="32" t="n"/>
+      <c r="H37" s="15" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I37" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J37" s="15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K37" s="15" t="inlineStr"/>
+      <c r="L37" s="32">
+        <f>IF(COUNTIF($B$5:B37,B37)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="18" t="inlineStr">
+        <is>
+          <t>EX-000021</t>
+        </is>
+      </c>
+      <c r="B38" s="18" t="inlineStr"/>
+      <c r="C38" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="D38" s="18" t="inlineStr">
+        <is>
+          <t>PO-523</t>
+        </is>
+      </c>
+      <c r="E38" s="18" t="inlineStr">
+        <is>
+          <t>P-9023A</t>
+        </is>
+      </c>
+      <c r="F38" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G38" s="33" t="n"/>
+      <c r="H38" s="18" t="inlineStr">
+        <is>
+          <t>Value Difference</t>
+        </is>
+      </c>
+      <c r="I38" s="18" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J38" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="K38" s="18" t="inlineStr"/>
+      <c r="L38" s="33">
+        <f>IF(COUNTIF($B$5:B38,B38)=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:K20"/>
+  <autoFilter ref="A4:K38"/>
   <mergeCells count="2">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A1:L1"/>
@@ -2577,19 +3402,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:S8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="35" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.5" customHeight="1">
@@ -2609,50 +3443,95 @@
     <row r="4" ht="27.75" customHeight="1">
       <c r="A4" s="37" t="inlineStr">
         <is>
+          <t>NORM_DOCUMENT NUMBER</t>
+        </is>
+      </c>
+      <c r="B4" s="37" t="inlineStr">
+        <is>
+          <t>BASE AMOUNT</t>
+        </is>
+      </c>
+      <c r="C4" s="37" t="inlineStr">
+        <is>
+          <t>GROSS AMOUNT</t>
+        </is>
+      </c>
+      <c r="D4" s="37" t="inlineStr">
+        <is>
           <t>DOCUMENT NUMBER</t>
         </is>
       </c>
-      <c r="B4" s="37" t="inlineStr">
+      <c r="E4" s="37" t="inlineStr">
         <is>
           <t>POSTING DATE</t>
         </is>
       </c>
-      <c r="C4" s="37" t="inlineStr">
+      <c r="F4" s="37" t="inlineStr">
         <is>
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="D4" s="37" t="inlineStr">
-        <is>
-          <t>BASE AMOUNT</t>
-        </is>
-      </c>
-      <c r="E4" s="37" t="inlineStr">
+      <c r="G4" s="37" t="inlineStr">
         <is>
           <t>TAX AMOUNT</t>
         </is>
       </c>
-      <c r="F4" s="37" t="inlineStr">
-        <is>
-          <t>GROSS AMOUNT</t>
-        </is>
-      </c>
-      <c r="G4" s="37" t="inlineStr">
+      <c r="H4" s="37" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
       </c>
-      <c r="H4" s="37" t="inlineStr">
+      <c r="I4" s="37" t="inlineStr">
         <is>
           <t>PORTAL REFERENCE</t>
         </is>
       </c>
-      <c r="I4" s="37" t="inlineStr">
+      <c r="J4" s="37" t="inlineStr">
         <is>
           <t>CATEGORY</t>
         </is>
       </c>
-      <c r="J4" s="37" t="inlineStr">
+      <c r="K4" s="37" t="inlineStr">
+        <is>
+          <t>__SOURCE_FILE__</t>
+        </is>
+      </c>
+      <c r="L4" s="37" t="inlineStr">
+        <is>
+          <t>__SOURCE_SHEET__</t>
+        </is>
+      </c>
+      <c r="M4" s="37" t="inlineStr">
+        <is>
+          <t>__SOURCE_ROW__</t>
+        </is>
+      </c>
+      <c r="N4" s="37" t="inlineStr">
+        <is>
+          <t>NORM_POSTING DATE</t>
+        </is>
+      </c>
+      <c r="O4" s="37" t="inlineStr">
+        <is>
+          <t>NORM_SUPPLIER</t>
+        </is>
+      </c>
+      <c r="P4" s="37" t="inlineStr">
+        <is>
+          <t>NORM_BASE AMOUNT</t>
+        </is>
+      </c>
+      <c r="Q4" s="37" t="inlineStr">
+        <is>
+          <t>NORM_GROSS AMOUNT</t>
+        </is>
+      </c>
+      <c r="R4" s="37" t="inlineStr">
+        <is>
+          <t>__GROUP_COUNT__</t>
+        </is>
+      </c>
+      <c r="S4" s="37" t="inlineStr">
         <is>
           <t>RecliQ_Universal_Reconciliation_Master_Test - portal.xlsx Row</t>
         </is>
@@ -2661,91 +3540,323 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
+          <t>INV1019A</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="n">
+        <v>18000</v>
+      </c>
+      <c r="C5" s="31" t="n">
+        <v>21240</v>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
           <t>INV1019-A</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>Zenith Industries</t>
         </is>
       </c>
-      <c r="D5" s="34" t="n">
+      <c r="G5" s="31" t="n">
+        <v>3240</v>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>Posted</t>
+        </is>
+      </c>
+      <c r="I5" s="15" t="inlineStr">
+        <is>
+          <t>P-9019A</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>Manufacturing</t>
+        </is>
+      </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>RecliQ_Universal_Reconciliation_Master_Test - portal.xlsx</t>
+        </is>
+      </c>
+      <c r="L5" s="15" t="inlineStr">
+        <is>
+          <t>Portal</t>
+        </is>
+      </c>
+      <c r="M5" s="31" t="n">
+        <v>20</v>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="O5" s="15" t="inlineStr">
+        <is>
+          <t>zenith industries</t>
+        </is>
+      </c>
+      <c r="P5" s="31" t="n">
         <v>18000</v>
       </c>
-      <c r="E5" s="34" t="n">
-        <v>3240</v>
-      </c>
-      <c r="F5" s="34" t="n">
+      <c r="Q5" s="31" t="n">
         <v>21240</v>
       </c>
-      <c r="G5" s="15" t="inlineStr">
-        <is>
-          <t>Posted</t>
-        </is>
-      </c>
-      <c r="H5" s="34" t="n">
-        <v>-9019</v>
-      </c>
-      <c r="I5" s="15" t="inlineStr">
-        <is>
-          <t>Manufacturing</t>
-        </is>
-      </c>
-      <c r="J5" s="31" t="n">
+      <c r="R5" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" s="32" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="18" t="inlineStr">
         <is>
+          <t>INV1019B</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C6" s="34" t="n">
+        <v>14160</v>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
           <t>INV1019-B</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="F6" s="18" t="inlineStr">
         <is>
           <t>Zenith Industries</t>
         </is>
       </c>
-      <c r="D6" s="32" t="n">
+      <c r="G6" s="34" t="n">
+        <v>2160</v>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Posted</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>P-9019B</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Manufacturing</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>RecliQ_Universal_Reconciliation_Master_Test - portal.xlsx</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>Portal</t>
+        </is>
+      </c>
+      <c r="M6" s="34" t="n">
+        <v>21</v>
+      </c>
+      <c r="N6" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="O6" s="18" t="inlineStr">
+        <is>
+          <t>zenith industries</t>
+        </is>
+      </c>
+      <c r="P6" s="34" t="n">
         <v>12000</v>
       </c>
-      <c r="E6" s="32" t="n">
+      <c r="Q6" s="34" t="n">
+        <v>14160</v>
+      </c>
+      <c r="R6" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="S6" s="33" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>INV1023</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C7" s="31" t="n">
+        <v>14160</v>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>INV1023</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>23-Aug-2026</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>Duplicate Test Co</t>
+        </is>
+      </c>
+      <c r="G7" s="31" t="n">
         <v>2160</v>
       </c>
-      <c r="F6" s="32" t="n">
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>Posted</t>
+        </is>
+      </c>
+      <c r="I7" s="15" t="inlineStr">
+        <is>
+          <t>P-9023A</t>
+        </is>
+      </c>
+      <c r="J7" s="15" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="K7" s="15" t="inlineStr">
+        <is>
+          <t>RecliQ_Universal_Reconciliation_Master_Test - portal.xlsx</t>
+        </is>
+      </c>
+      <c r="L7" s="15" t="inlineStr">
+        <is>
+          <t>Portal</t>
+        </is>
+      </c>
+      <c r="M7" s="31" t="n">
+        <v>24</v>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>23-Aug-2026</t>
+        </is>
+      </c>
+      <c r="O7" s="15" t="inlineStr">
+        <is>
+          <t>duplicate test co</t>
+        </is>
+      </c>
+      <c r="P7" s="31" t="n">
+        <v>12000</v>
+      </c>
+      <c r="Q7" s="31" t="n">
         <v>14160</v>
       </c>
-      <c r="G6" s="18" t="inlineStr">
+      <c r="R7" s="15" t="n"/>
+      <c r="S7" s="15" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>INV1023</t>
+        </is>
+      </c>
+      <c r="B8" s="34" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C8" s="34" t="n">
+        <v>14160</v>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>INV1023</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>23-Aug-2026</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Duplicate Test Co</t>
+        </is>
+      </c>
+      <c r="G8" s="34" t="n">
+        <v>2160</v>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
         <is>
           <t>Posted</t>
         </is>
       </c>
-      <c r="H6" s="32" t="n">
-        <v>-9019</v>
-      </c>
-      <c r="I6" s="18" t="inlineStr">
-        <is>
-          <t>Manufacturing</t>
-        </is>
-      </c>
-      <c r="J6" s="33" t="n">
-        <v>21</v>
-      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>P-9023B</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>RecliQ_Universal_Reconciliation_Master_Test - portal.xlsx</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>Portal</t>
+        </is>
+      </c>
+      <c r="M8" s="34" t="n">
+        <v>25</v>
+      </c>
+      <c r="N8" s="18" t="inlineStr">
+        <is>
+          <t>23-Aug-2026</t>
+        </is>
+      </c>
+      <c r="O8" s="18" t="inlineStr">
+        <is>
+          <t>duplicate test co</t>
+        </is>
+      </c>
+      <c r="P8" s="34" t="n">
+        <v>12000</v>
+      </c>
+      <c r="Q8" s="34" t="n">
+        <v>14160</v>
+      </c>
+      <c r="R8" s="18" t="n"/>
+      <c r="S8" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A2:S2"/>
+    <mergeCell ref="A1:S1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -2761,18 +3872,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="35" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.5" customHeight="1">
@@ -2792,45 +3912,90 @@
     <row r="4" ht="27.75" customHeight="1">
       <c r="A4" s="37" t="inlineStr">
         <is>
+          <t>NORM_INVOICE NO</t>
+        </is>
+      </c>
+      <c r="B4" s="37" t="inlineStr">
+        <is>
+          <t>TAXABLE VALUE</t>
+        </is>
+      </c>
+      <c r="C4" s="37" t="inlineStr">
+        <is>
+          <t>TOTAL BOOK VALUE</t>
+        </is>
+      </c>
+      <c r="D4" s="37" t="inlineStr">
+        <is>
           <t>INVOICE NO</t>
         </is>
       </c>
-      <c r="B4" s="37" t="inlineStr">
+      <c r="E4" s="37" t="inlineStr">
         <is>
           <t>INVOICE DATE</t>
         </is>
       </c>
-      <c r="C4" s="37" t="inlineStr">
+      <c r="F4" s="37" t="inlineStr">
         <is>
           <t>VENDOR NAME</t>
         </is>
       </c>
-      <c r="D4" s="37" t="inlineStr">
-        <is>
-          <t>TAXABLE VALUE</t>
-        </is>
-      </c>
-      <c r="E4" s="37" t="inlineStr">
+      <c r="G4" s="37" t="inlineStr">
         <is>
           <t>GST</t>
         </is>
       </c>
-      <c r="F4" s="37" t="inlineStr">
-        <is>
-          <t>TOTAL BOOK VALUE</t>
-        </is>
-      </c>
-      <c r="G4" s="37" t="inlineStr">
+      <c r="H4" s="37" t="inlineStr">
         <is>
           <t>DEPARTMENT</t>
         </is>
       </c>
-      <c r="H4" s="37" t="inlineStr">
+      <c r="I4" s="37" t="inlineStr">
         <is>
           <t>PO REFERENCE</t>
         </is>
       </c>
-      <c r="I4" s="37" t="inlineStr">
+      <c r="J4" s="37" t="inlineStr">
+        <is>
+          <t>__SOURCE_FILE__</t>
+        </is>
+      </c>
+      <c r="K4" s="37" t="inlineStr">
+        <is>
+          <t>__SOURCE_SHEET__</t>
+        </is>
+      </c>
+      <c r="L4" s="37" t="inlineStr">
+        <is>
+          <t>__SOURCE_ROW__</t>
+        </is>
+      </c>
+      <c r="M4" s="37" t="inlineStr">
+        <is>
+          <t>NORM_INVOICE DATE</t>
+        </is>
+      </c>
+      <c r="N4" s="37" t="inlineStr">
+        <is>
+          <t>NORM_VENDOR NAME</t>
+        </is>
+      </c>
+      <c r="O4" s="37" t="inlineStr">
+        <is>
+          <t>NORM_TAXABLE VALUE</t>
+        </is>
+      </c>
+      <c r="P4" s="37" t="inlineStr">
+        <is>
+          <t>NORM_TOTAL BOOK VALUE</t>
+        </is>
+      </c>
+      <c r="Q4" s="37" t="inlineStr">
+        <is>
+          <t>__GROUP_COUNT__</t>
+        </is>
+      </c>
+      <c r="R4" s="37" t="inlineStr">
         <is>
           <t>RecliQ_Universal_Reconciliation_Master_Test - Book.xlsx Row</t>
         </is>
@@ -2839,81 +4004,159 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
+          <t>INV1019</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C5" s="31" t="n">
+        <v>35400</v>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
           <t>INV/1019</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>Zenith Industries</t>
         </is>
       </c>
-      <c r="D5" s="34" t="n">
+      <c r="G5" s="31" t="n">
+        <v>5400</v>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="I5" s="15" t="inlineStr">
+        <is>
+          <t>PO-519</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>RecliQ_Universal_Reconciliation_Master_Test - Book.xlsx</t>
+        </is>
+      </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>Books</t>
+        </is>
+      </c>
+      <c r="L5" s="31" t="n">
+        <v>20</v>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>19/08/2026</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>zenith industries</t>
+        </is>
+      </c>
+      <c r="O5" s="31" t="n">
         <v>30000</v>
       </c>
-      <c r="E5" s="34" t="n">
-        <v>5400</v>
-      </c>
-      <c r="F5" s="34" t="n">
+      <c r="P5" s="31" t="n">
         <v>35400</v>
       </c>
-      <c r="G5" s="15" t="inlineStr">
-        <is>
-          <t>Operations</t>
-        </is>
-      </c>
-      <c r="H5" s="34" t="n">
-        <v>-519</v>
-      </c>
-      <c r="I5" s="31" t="n">
+      <c r="Q5" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="R5" s="32" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="18" t="inlineStr">
         <is>
+          <t>INV1021</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C6" s="34" t="n">
+        <v>5900</v>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
           <t>INV/1021</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>21-08-2026</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="F6" s="18" t="inlineStr">
         <is>
           <t>Missing From Portal Ltd</t>
         </is>
       </c>
-      <c r="D6" s="32" t="n">
+      <c r="G6" s="34" t="n">
+        <v>900</v>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>PO-521</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>RecliQ_Universal_Reconciliation_Master_Test - Book.xlsx</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Books</t>
+        </is>
+      </c>
+      <c r="L6" s="34" t="n">
+        <v>22</v>
+      </c>
+      <c r="M6" s="18" t="inlineStr">
+        <is>
+          <t>21-08-2026</t>
+        </is>
+      </c>
+      <c r="N6" s="18" t="inlineStr">
+        <is>
+          <t>missing from portal ltd</t>
+        </is>
+      </c>
+      <c r="O6" s="34" t="n">
         <v>5000</v>
       </c>
-      <c r="E6" s="32" t="n">
-        <v>900</v>
-      </c>
-      <c r="F6" s="32" t="n">
+      <c r="P6" s="34" t="n">
         <v>5900</v>
       </c>
-      <c r="G6" s="18" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="H6" s="32" t="n">
-        <v>-521</v>
-      </c>
-      <c r="I6" s="33" t="n">
+      <c r="Q6" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" s="33" t="n">
         <v>22</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -2929,7 +4172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2993,58 +4236,50 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>INV/1002</t>
-        </is>
-      </c>
+      <c r="A5" s="15" t="inlineStr"/>
       <c r="B5" s="15" t="inlineStr">
         <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>PO-501</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>P-9001</t>
+        </is>
+      </c>
+      <c r="E5" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F5" s="32" t="n"/>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr"/>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
           <t>INVOICE DATE</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>02-Aug-2026</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="E5" s="31" t="n"/>
-      <c r="F5" s="31" t="n"/>
-      <c r="G5" s="15" t="inlineStr">
-        <is>
-          <t>Mismatch</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>INV/1004</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>INVOICE DATE</t>
-        </is>
-      </c>
-      <c r="C6" s="18" t="inlineStr">
-        <is>
-          <t>2026/08/04</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>04/08/2026</t>
-        </is>
-      </c>
-      <c r="E6" s="32" t="n">
-        <v>16178778</v>
-      </c>
+      <c r="E6" s="33" t="n"/>
       <c r="F6" s="33" t="n"/>
       <c r="G6" s="18" t="inlineStr">
         <is>
@@ -3053,28 +4288,26 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>INV/1005</t>
-        </is>
-      </c>
+      <c r="A7" s="15" t="inlineStr"/>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>INVOICE DATE</t>
+          <t>PO REFERENCE</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>05-08-2026</t>
+          <t>PO-502</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="E7" s="31" t="n"/>
-      <c r="F7" s="31" t="n"/>
+          <t>P-9002</t>
+        </is>
+      </c>
+      <c r="E7" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F7" s="32" t="n"/>
       <c r="G7" s="15" t="inlineStr">
         <is>
           <t>Mismatch</t>
@@ -3082,27 +4315,25 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>INV/1006</t>
-        </is>
-      </c>
+      <c r="A8" s="18" t="inlineStr"/>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>INVOICE DATE</t>
+          <t>PO REFERENCE</t>
         </is>
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>PO-503</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>06-Aug-2026</t>
-        </is>
-      </c>
-      <c r="E8" s="33" t="n"/>
+          <t>P-9003</t>
+        </is>
+      </c>
+      <c r="E8" s="34" t="n">
+        <v>8500</v>
+      </c>
       <c r="F8" s="33" t="n"/>
       <c r="G8" s="18" t="inlineStr">
         <is>
@@ -3111,11 +4342,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>INV/1007</t>
-        </is>
-      </c>
+      <c r="A9" s="15" t="inlineStr"/>
       <c r="B9" s="15" t="inlineStr">
         <is>
           <t>INVOICE DATE</t>
@@ -3123,18 +4350,18 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>2026/08/04</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>2026/08/07</t>
-        </is>
-      </c>
-      <c r="E9" s="34" t="n">
-        <v>-13178781</v>
-      </c>
-      <c r="F9" s="31" t="n"/>
+          <t>04/08/2026</t>
+        </is>
+      </c>
+      <c r="E9" s="31" t="n">
+        <v>16178778</v>
+      </c>
+      <c r="F9" s="32" t="n"/>
       <c r="G9" s="15" t="inlineStr">
         <is>
           <t>Mismatch</t>
@@ -3142,27 +4369,25 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>INV/1008</t>
-        </is>
-      </c>
+      <c r="A10" s="18" t="inlineStr"/>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>INVOICE DATE</t>
+          <t>PO REFERENCE</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>PO-504</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
         <is>
-          <t>08-08-2026</t>
-        </is>
-      </c>
-      <c r="E10" s="33" t="n"/>
+          <t>P-9004</t>
+        </is>
+      </c>
+      <c r="E10" s="34" t="n">
+        <v>8500</v>
+      </c>
       <c r="F10" s="33" t="n"/>
       <c r="G10" s="18" t="inlineStr">
         <is>
@@ -3171,11 +4396,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
-        <is>
-          <t>INV/1009</t>
-        </is>
-      </c>
+      <c r="A11" s="15" t="inlineStr"/>
       <c r="B11" s="15" t="inlineStr">
         <is>
           <t>INVOICE DATE</t>
@@ -3183,16 +4404,16 @@
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>09-Aug-2026</t>
+          <t>05-08-2026</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="E11" s="31" t="n"/>
-      <c r="F11" s="31" t="n"/>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="n"/>
+      <c r="F11" s="32" t="n"/>
       <c r="G11" s="15" t="inlineStr">
         <is>
           <t>Mismatch</t>
@@ -3200,27 +4421,25 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>INV/1012</t>
-        </is>
-      </c>
+      <c r="A12" s="18" t="inlineStr"/>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>INVOICE DATE</t>
+          <t>PO REFERENCE</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>PO-505</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>12-Aug-2026</t>
-        </is>
-      </c>
-      <c r="E12" s="33" t="n"/>
+          <t>P-9005</t>
+        </is>
+      </c>
+      <c r="E12" s="34" t="n">
+        <v>8500</v>
+      </c>
       <c r="F12" s="33" t="n"/>
       <c r="G12" s="18" t="inlineStr">
         <is>
@@ -3229,11 +4448,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>INV/1017</t>
-        </is>
-      </c>
+      <c r="A13" s="15" t="inlineStr"/>
       <c r="B13" s="15" t="inlineStr">
         <is>
           <t>INVOICE DATE</t>
@@ -3241,16 +4456,16 @@
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>17-Aug-2026</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="E13" s="31" t="n"/>
-      <c r="F13" s="31" t="n"/>
+          <t>06-Aug-2026</t>
+        </is>
+      </c>
+      <c r="E13" s="32" t="n"/>
+      <c r="F13" s="32" t="n"/>
       <c r="G13" s="15" t="inlineStr">
         <is>
           <t>Mismatch</t>
@@ -3258,27 +4473,25 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>INV/1020</t>
-        </is>
-      </c>
+      <c r="A14" s="18" t="inlineStr"/>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>INVOICE DATE</t>
+          <t>PO REFERENCE</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>PO-506</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>20-Aug-2026</t>
-        </is>
-      </c>
-      <c r="E14" s="33" t="n"/>
+          <t>P-9006</t>
+        </is>
+      </c>
+      <c r="E14" s="34" t="n">
+        <v>8500</v>
+      </c>
       <c r="F14" s="33" t="n"/>
       <c r="G14" s="18" t="inlineStr">
         <is>
@@ -3287,174 +4500,632 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>INV/1022</t>
-        </is>
-      </c>
+      <c r="A15" s="15" t="inlineStr"/>
       <c r="B15" s="15" t="inlineStr">
         <is>
+          <t>INVOICE DATE</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>2026/08/07</t>
+        </is>
+      </c>
+      <c r="E15" s="31" t="n">
+        <v>-13178781</v>
+      </c>
+      <c r="F15" s="32" t="n"/>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr"/>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>PO-507</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>P-9007</t>
+        </is>
+      </c>
+      <c r="E16" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F16" s="33" t="n"/>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr"/>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>INVOICE DATE</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>08-08-2026</t>
+        </is>
+      </c>
+      <c r="E17" s="32" t="n"/>
+      <c r="F17" s="32" t="n"/>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr"/>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>PO-508</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>P-9008</t>
+        </is>
+      </c>
+      <c r="E18" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F18" s="33" t="n"/>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr"/>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>INVOICE DATE</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>09-Aug-2026</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="E19" s="32" t="n"/>
+      <c r="F19" s="32" t="n"/>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr"/>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>PO-509</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>P-9009</t>
+        </is>
+      </c>
+      <c r="E20" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F20" s="33" t="n"/>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr"/>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>PO-510</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>P-9010</t>
+        </is>
+      </c>
+      <c r="E21" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F21" s="32" t="n"/>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr"/>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>PO-511</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>P-9011</t>
+        </is>
+      </c>
+      <c r="E22" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F22" s="33" t="n"/>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr"/>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>INVOICE DATE</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>12-Aug-2026</t>
+        </is>
+      </c>
+      <c r="E23" s="32" t="n"/>
+      <c r="F23" s="32" t="n"/>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr"/>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>PO-512</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>P-9012</t>
+        </is>
+      </c>
+      <c r="E24" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F24" s="33" t="n"/>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr"/>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>PO-513</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>P-9013</t>
+        </is>
+      </c>
+      <c r="E25" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F25" s="32" t="n"/>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr"/>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>PO-514</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>P-9014</t>
+        </is>
+      </c>
+      <c r="E26" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F26" s="33" t="n"/>
+      <c r="G26" s="18" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr"/>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>PO-515</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>P-9015</t>
+        </is>
+      </c>
+      <c r="E27" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F27" s="32" t="n"/>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr"/>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C28" s="18" t="inlineStr">
+        <is>
+          <t>PO-516</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>P-9016</t>
+        </is>
+      </c>
+      <c r="E28" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F28" s="33" t="n"/>
+      <c r="G28" s="18" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr"/>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>INVOICE DATE</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>17-Aug-2026</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="E29" s="32" t="n"/>
+      <c r="F29" s="32" t="n"/>
+      <c r="G29" s="15" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr"/>
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
+          <t>PO-517</t>
+        </is>
+      </c>
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>P-9017</t>
+        </is>
+      </c>
+      <c r="E30" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F30" s="33" t="n"/>
+      <c r="G30" s="18" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr"/>
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>PO-518</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>P-9018</t>
+        </is>
+      </c>
+      <c r="E31" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F31" s="32" t="n"/>
+      <c r="G31" s="15" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr"/>
+      <c r="B32" s="18" t="inlineStr">
+        <is>
+          <t>INVOICE DATE</t>
+        </is>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="D32" s="18" t="inlineStr">
+        <is>
+          <t>20-Aug-2026</t>
+        </is>
+      </c>
+      <c r="E32" s="33" t="n"/>
+      <c r="F32" s="33" t="n"/>
+      <c r="G32" s="18" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr"/>
+      <c r="B33" s="15" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>PO-520</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>P-9020</t>
+        </is>
+      </c>
+      <c r="E33" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F33" s="32" t="n"/>
+      <c r="G33" s="15" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr"/>
+      <c r="B34" s="18" t="inlineStr">
+        <is>
           <t>TAXABLE VALUE</t>
         </is>
       </c>
-      <c r="C15" s="34" t="n">
+      <c r="C34" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="34" t="n">
+      <c r="D34" s="34" t="n">
         <v>4000</v>
       </c>
-      <c r="E15" s="34" t="n">
+      <c r="E34" s="34" t="n">
         <v>-4000</v>
       </c>
-      <c r="F15" s="35" t="n">
+      <c r="F34" s="35" t="n">
         <v>-1</v>
       </c>
-      <c r="G15" s="15" t="inlineStr">
+      <c r="G34" s="18" t="inlineStr">
         <is>
           <t>Mismatch</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>INV/1022</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr"/>
+      <c r="B35" s="15" t="inlineStr">
         <is>
           <t>GST</t>
         </is>
       </c>
-      <c r="C16" s="32" t="n">
+      <c r="C35" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="32" t="n">
+      <c r="D35" s="31" t="n">
         <v>720</v>
       </c>
-      <c r="E16" s="32" t="n">
+      <c r="E35" s="31" t="n">
         <v>-720</v>
       </c>
-      <c r="F16" s="36" t="n">
+      <c r="F35" s="36" t="n">
         <v>-1</v>
       </c>
-      <c r="G16" s="18" t="inlineStr">
+      <c r="G35" s="15" t="inlineStr">
         <is>
           <t>Mismatch</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>INV/1022</t>
-        </is>
-      </c>
-      <c r="B17" s="15" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="18" t="inlineStr"/>
+      <c r="B36" s="18" t="inlineStr">
         <is>
           <t>TOTAL BOOK VALUE</t>
         </is>
       </c>
-      <c r="C17" s="34" t="n">
+      <c r="C36" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="34" t="n">
+      <c r="D36" s="34" t="n">
         <v>4720</v>
       </c>
-      <c r="E17" s="34" t="n">
+      <c r="E36" s="34" t="n">
         <v>-4720</v>
       </c>
-      <c r="F17" s="35" t="n">
+      <c r="F36" s="35" t="n">
         <v>-1</v>
       </c>
-      <c r="G17" s="15" t="inlineStr">
+      <c r="G36" s="18" t="inlineStr">
         <is>
           <t>Mismatch</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>INV/1023</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>TAXABLE VALUE</t>
-        </is>
-      </c>
-      <c r="C18" s="32" t="n">
-        <v>12000</v>
-      </c>
-      <c r="D18" s="32" t="n">
-        <v>24000</v>
-      </c>
-      <c r="E18" s="32" t="n">
-        <v>-12000</v>
-      </c>
-      <c r="F18" s="36" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="G18" s="18" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr"/>
+      <c r="B37" s="15" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>PO-522</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>P-9022</t>
+        </is>
+      </c>
+      <c r="E37" s="31" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F37" s="32" t="n"/>
+      <c r="G37" s="15" t="inlineStr">
         <is>
           <t>Mismatch</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>INV/1023</t>
-        </is>
-      </c>
-      <c r="B19" s="15" t="inlineStr">
-        <is>
-          <t>GST</t>
-        </is>
-      </c>
-      <c r="C19" s="34" t="n">
-        <v>2160</v>
-      </c>
-      <c r="D19" s="34" t="n">
-        <v>4320</v>
-      </c>
-      <c r="E19" s="34" t="n">
-        <v>-2160</v>
-      </c>
-      <c r="F19" s="35" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="G19" s="15" t="inlineStr">
-        <is>
-          <t>Mismatch</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>INV/1023</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>TOTAL BOOK VALUE</t>
-        </is>
-      </c>
-      <c r="C20" s="32" t="n">
-        <v>14160</v>
-      </c>
-      <c r="D20" s="32" t="n">
-        <v>28320</v>
-      </c>
-      <c r="E20" s="32" t="n">
-        <v>-14160</v>
-      </c>
-      <c r="F20" s="36" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="G20" s="18" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="18" t="inlineStr"/>
+      <c r="B38" s="18" t="inlineStr">
+        <is>
+          <t>PO REFERENCE</t>
+        </is>
+      </c>
+      <c r="C38" s="18" t="inlineStr">
+        <is>
+          <t>PO-523</t>
+        </is>
+      </c>
+      <c r="D38" s="18" t="inlineStr">
+        <is>
+          <t>P-9023A</t>
+        </is>
+      </c>
+      <c r="E38" s="34" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F38" s="33" t="n"/>
+      <c r="G38" s="18" t="inlineStr">
         <is>
           <t>Mismatch</t>
         </is>
@@ -3529,11 +5200,11 @@
         </is>
       </c>
       <c r="B5" s="38">
-        <f>COUNTA('03 Matched Records'!C5:C5)+SUM('02 Exceptions'!L5:L20)+COUNTA('05 Missing - RecliQ_Universal_R'!A5:A6)</f>
+        <f>COUNTA('03 Matched Records'!C5:C5)+SUM('02 Exceptions'!L5:L38)+COUNTA('05 Missing - RecliQ_Universal_R'!A5:A6)</f>
         <v/>
       </c>
       <c r="C5" s="38">
-        <f>COUNTA('03 Matched Records'!C5:C5)+SUM('02 Exceptions'!L5:L20)+COUNTA('04 Missing - RecliQ_Universal_R'!A5:A6)</f>
+        <f>COUNTA('03 Matched Records'!C5:C5)+SUM('02 Exceptions'!L5:L38)+COUNTA('04 Missing - RecliQ_Universal_R'!A5:A8)</f>
         <v/>
       </c>
       <c r="D5" s="39">
@@ -3567,11 +5238,11 @@
         </is>
       </c>
       <c r="B7" s="38">
-        <f>SUM('02 Exceptions'!L5:L20)</f>
+        <f>SUM('02 Exceptions'!L5:L38)</f>
         <v/>
       </c>
       <c r="C7" s="38">
-        <f>SUM('02 Exceptions'!L5:L20)</f>
+        <f>SUM('02 Exceptions'!L5:L38)</f>
         <v/>
       </c>
       <c r="D7" s="39">
@@ -3586,7 +5257,7 @@
         </is>
       </c>
       <c r="B8" s="40">
-        <f>COUNTA('04 Missing - RecliQ_Universal_R'!A5:A6)</f>
+        <f>COUNTA('04 Missing - RecliQ_Universal_R'!A5:A8)</f>
         <v/>
       </c>
       <c r="C8" s="40" t="inlineStr">

</xml_diff>